<commit_message>
GĐ 1-2: Cấu trúc thư mục theo chức năng (user, project, task, comment).
</commit_message>
<xml_diff>
--- a/Schedule-Note.xlsx
+++ b/Schedule-Note.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\task-manager-laravel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECCE23B7-D72B-4423-97DE-EA0F8F6A3C1F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8508CD66-4B79-46CA-9ED9-AFFFFA2EEA7E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="141">
   <si>
     <t>STT</t>
   </si>
@@ -121,9 +121,6 @@
   </si>
   <si>
     <t>Ghi chú</t>
-  </si>
-  <si>
-    <t>Gợi ý cấu trúc thư mục Laravel (theo chức năng)</t>
   </si>
   <si>
     <t>- Tạo project Laravel
@@ -148,18 +145,332 @@
     <t>Libraries/Lệnh</t>
   </si>
   <si>
-    <t>laravel new task-manager-laravel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5/7
-</t>
+    <t>5/7
+5/7</t>
+  </si>
+  <si>
+    <t>laravel new task-manager-laravel
+php artisan make:model Task -a</t>
+  </si>
+  <si>
+    <t>app</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    ├── Http</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   ├── Controllers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   │   ├── Comment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   │   │   └── CommentController.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   │   ├── Project</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   │   │   └── ProjectController.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   │   ├── Task</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   │   │   └── TaskController.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   │   ├── User</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   │   │   └── UserController.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   └── Requests</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │       ├── Comment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │       │   ├── StoreCommentRequest.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │       │   └── UpdateCommentRequest.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │       ├── Project</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │       │   ├── StoreProjectRequest.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │       │   └── UpdateProjectRequest.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │       ├── Task</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │       │   ├── StoreTaskRequest.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │       │   └── UpdateTaskRequest.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │       └── User</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │           ├── StoreUserRequest.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │           └── UpdateUserRequest.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    ├── Models</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   ├── Comment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   │   └── Comment.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   ├── Default</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   │   └── User.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   ├── Project</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   │   └── Project.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   ├── Task</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   │   └── Task.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   └── User</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │       └── User.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    ├── Policies</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   │   └── CommentPolicy.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   │   └── ProjectPolicy.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   │   └── TaskPolicy.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │       └── UserPolicy.php</t>
+  </si>
+  <si>
+    <t>Cấu trúc thư mục Laravel (theo chức năng)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 
+tạo 8 file (folder default chứa file mặc định của laravel)</t>
+  </si>
+  <si>
+    <t>database</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    ├── factories</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   ├── default</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   │   └── UserFactory.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   ├── CommentFactory.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   ├── ProjectFactory.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   ├── TaskFactory.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   └── UserFactory.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    ├── migrations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   │   ├── 0001_01_01_000000_create_users_table.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   │   ├── 0001_01_01_000001_create_cache_table.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   │   └── 0001_01_01_000002_create_jobs_table.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   ├── 2025_07_05_021021_create_tasks_table.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   ├── 2025_07_05_022217_create_users_table.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   ├── 2025_07_05_022238_create_projects_table.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   └── 2025_07_05_022249_create_comments_table.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    ├── seeders</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   │   └── DatabaseSeeder.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   ├── CommentSeeder.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   ├── ProjectSeeder.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   ├── TaskSeeder.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   └── UserSeeder.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    └── .gitignore</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   │   ├── Controller.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   │   └── DashboardController.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    ├── Providers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   └── AppServiceProvider.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    └── Services</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        ├── Comment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        │   └── CommentService.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        ├── Project</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        │   └── ProjectService.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        ├── Task</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        │   └── TaskService.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        └── User</t>
+  </si>
+  <si>
+    <t xml:space="preserve">            └── UserService.php</t>
+  </si>
+  <si>
+    <t>views</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    ├── comments</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   ├── _form.blade.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   ├── create.blade.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   ├── edit.blade.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   ├── index.blade.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   └── show.blade.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    ├── dashboard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   └── index.blade.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    ├── layouts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   └── master.blade.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    ├── partials</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   └── _test.blade.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    ├── projects</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    ├── tasks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    ├── users</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    └── welcome.blade.php</t>
+  </si>
+  <si>
+    <t>routes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    ├── web</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   ├── comment.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   ├── dashboard.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   ├── project.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   ├── task.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    │   └── user.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    ├── console.php</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    └── web.php</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -218,6 +529,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="20"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -260,7 +578,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -300,6 +618,8 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="16" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -312,22 +632,22 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="16" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="16" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -424,6 +744,50 @@
         <a:xfrm>
           <a:off x="4324350" y="781050"/>
           <a:ext cx="6081287" cy="5296359"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>247650</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>1630207</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>58004</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DE865C10-DB21-4158-8A03-6527E3DF6DA3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10620375" y="933450"/>
+          <a:ext cx="10259857" cy="6115904"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -732,36 +1096,36 @@
     <col min="8" max="8" width="32.7109375" style="8" customWidth="1"/>
     <col min="9" max="9" width="10.140625" style="8" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="31.28515625" style="8" customWidth="1"/>
-    <col min="11" max="11" width="8.5703125" style="8" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="49.5703125" style="8" customWidth="1"/>
     <col min="12" max="16384" width="9.140625" style="8"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:11" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
-      <c r="D3" s="18" t="s">
+      <c r="D3" s="20" t="s">
         <v>22</v>
       </c>
-      <c r="E3" s="18"/>
+      <c r="E3" s="20"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
-      <c r="D4" s="18" t="s">
+      <c r="D4" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="18"/>
+      <c r="E4" s="20"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -769,12 +1133,12 @@
       <c r="C5" s="1"/>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
-      <c r="H5" s="19" t="s">
+      <c r="H5" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="I5" s="20"/>
-      <c r="J5" s="20"/>
-      <c r="K5" s="20"/>
+      <c r="I5" s="22"/>
+      <c r="J5" s="22"/>
+      <c r="K5" s="22"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
@@ -805,7 +1169,7 @@
         <v>28</v>
       </c>
       <c r="J6" s="10" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="K6" s="10" t="s">
         <v>29</v>
@@ -819,24 +1183,26 @@
         <v>5</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E7" s="7" t="s">
         <v>25</v>
       </c>
       <c r="H7" s="14" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="I7" s="15" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="J7" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="K7" s="3"/>
+      <c r="K7" s="23" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="8" spans="1:11" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
@@ -951,7 +1317,7 @@
         <v>20</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D13" s="3" t="s">
         <v>8</v>
@@ -1000,76 +1366,664 @@
   <dimension ref="B4:P166"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="21"/>
-    <col min="2" max="2" width="9.85546875" style="21" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="44.28515625" style="21" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="78.140625" style="21" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.140625" style="21" customWidth="1"/>
-    <col min="6" max="6" width="26.42578125" style="21" bestFit="1" customWidth="1"/>
-    <col min="7" max="14" width="9.140625" style="21"/>
-    <col min="15" max="15" width="33.5703125" style="21" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="78.140625" style="21" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.140625" style="21"/>
+    <col min="1" max="1" width="9.140625" style="18"/>
+    <col min="2" max="2" width="9.85546875" style="18" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="53.85546875" style="18" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="78.140625" style="18" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.140625" style="18" customWidth="1"/>
+    <col min="6" max="6" width="26.42578125" style="18" bestFit="1" customWidth="1"/>
+    <col min="7" max="14" width="9.140625" style="18"/>
+    <col min="15" max="15" width="33.5703125" style="18" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="78.140625" style="18" bestFit="1" customWidth="1"/>
+    <col min="17" max="16384" width="9.140625" style="18"/>
   </cols>
   <sheetData>
-    <row r="4" spans="2:16" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
+    <row r="4" spans="2:15" s="29" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
       <c r="B4" s="16">
         <v>45843</v>
       </c>
-      <c r="O4" s="16"/>
-    </row>
-    <row r="5" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="C5" s="22" t="s">
-        <v>30</v>
-      </c>
-      <c r="O5" s="22"/>
-      <c r="P5" s="22"/>
-    </row>
-    <row r="12" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="O12" s="22"/>
-    </row>
-    <row r="24" spans="15:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="O24" s="23"/>
-      <c r="P24" s="23"/>
-    </row>
-    <row r="25" spans="15:16" x14ac:dyDescent="0.25">
-      <c r="O25" s="23"/>
-      <c r="P25" s="23"/>
-    </row>
-    <row r="108" spans="2:7" ht="26.25" x14ac:dyDescent="0.4">
+      <c r="O4" s="30"/>
+    </row>
+    <row r="5" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="C5" s="17" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="6" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="C6" s="17" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="7" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="C7" s="18" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="8" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="C8" s="18" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="9" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="C9" s="18" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="10" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="C10" s="18" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="11" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="C11" s="18" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="12" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="C12" s="18" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="13" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="C13" s="18" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="14" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="C14" s="18" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="15" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="C15" s="18" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="16" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="C16" s="18" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="17" spans="3:16" x14ac:dyDescent="0.25">
+      <c r="C17" s="18" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="18" spans="3:16" x14ac:dyDescent="0.25">
+      <c r="C18" s="18" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="19" spans="3:16" x14ac:dyDescent="0.25">
+      <c r="C19" s="18" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="20" spans="3:16" x14ac:dyDescent="0.25">
+      <c r="C20" s="18" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="21" spans="3:16" x14ac:dyDescent="0.25">
+      <c r="C21" s="18" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="22" spans="3:16" x14ac:dyDescent="0.25">
+      <c r="C22" s="18" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="23" spans="3:16" x14ac:dyDescent="0.25">
+      <c r="C23" s="18" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="24" spans="3:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C24" s="18" t="s">
+        <v>53</v>
+      </c>
+      <c r="O24" s="26"/>
+      <c r="P24" s="26"/>
+    </row>
+    <row r="25" spans="3:16" x14ac:dyDescent="0.25">
+      <c r="C25" s="18" t="s">
+        <v>54</v>
+      </c>
+      <c r="O25" s="26"/>
+      <c r="P25" s="26"/>
+    </row>
+    <row r="26" spans="3:16" x14ac:dyDescent="0.25">
+      <c r="C26" s="18" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="27" spans="3:16" x14ac:dyDescent="0.25">
+      <c r="C27" s="18" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="28" spans="3:16" x14ac:dyDescent="0.25">
+      <c r="C28" s="18" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="29" spans="3:16" x14ac:dyDescent="0.25">
+      <c r="C29" s="18" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="30" spans="3:16" x14ac:dyDescent="0.25">
+      <c r="C30" s="18" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="31" spans="3:16" x14ac:dyDescent="0.25">
+      <c r="C31" s="18" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="32" spans="3:16" x14ac:dyDescent="0.25">
+      <c r="C32" s="18" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="33" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C33" s="18" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="34" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C34" s="18" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="35" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C35" s="18" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="36" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C36" s="18" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="37" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C37" s="18" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="38" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C38" s="18" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="39" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C39" s="18" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="40" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C40" s="18" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="41" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C41" s="18" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="42" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C42" s="18" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="43" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C43" s="18" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="44" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C44" s="18" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="45" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C45" s="18" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="46" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C46" s="18" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="47" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C47" s="18" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="48" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C48" s="18" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="49" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C49" s="18" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="50" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C50" s="18" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="51" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C51" s="18" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="52" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C52" s="18" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="53" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C53" s="18" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="54" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C54" s="18" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="55" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C55" s="18" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="56" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C56" s="18" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="57" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C57" s="18" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="58" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C58" s="18" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="59" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C59" s="18" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="60" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C60" s="18" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="61" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C61" s="18" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="62" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C62" s="18" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="64" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C64" s="17" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="65" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C65" s="18" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="66" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C66" s="18" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="67" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C67" s="18" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="68" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C68" s="18" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="69" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C69" s="18" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="70" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C70" s="18" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="71" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C71" s="18" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="72" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C72" s="18" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="73" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C73" s="18" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="74" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C74" s="18" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="75" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C75" s="18" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="76" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C76" s="18" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="77" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C77" s="18" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="78" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C78" s="18" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="79" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C79" s="18" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="80" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C80" s="18" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="81" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C81" s="18" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="82" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C82" s="18" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="83" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C83" s="18" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="84" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C84" s="18" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="85" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C85" s="18" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="86" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C86" s="18" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="87" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C87" s="18" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="88" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C88" s="18" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="90" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C90" s="17" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="91" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C91" s="18" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="92" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C92" s="18" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="93" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C93" s="18" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="94" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C94" s="18" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="95" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C95" s="18" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="96" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C96" s="18" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="97" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C97" s="18" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="98" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C98" s="18" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="99" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C99" s="18" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="100" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C100" s="18" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="101" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C101" s="18" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="102" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C102" s="18" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="103" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C103" s="18" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="104" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C104" s="18" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="105" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C105" s="18" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="106" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C106" s="18" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="107" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C107" s="18" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="108" spans="2:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B108" s="24"/>
-      <c r="C108" s="24"/>
-    </row>
-    <row r="109" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="C109" s="22"/>
-      <c r="D109" s="22"/>
-      <c r="F109" s="22"/>
-      <c r="G109" s="25"/>
+      <c r="C108" s="25" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="109" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C109" s="18" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="110" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C110" s="18" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="111" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C111" s="18" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="112" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C112" s="18" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="113" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C113" s="18" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="114" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C114" s="18" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="115" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C115" s="18" t="s">
+        <v>130</v>
+      </c>
     </row>
     <row r="116" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C116" s="22"/>
+      <c r="C116" s="18" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="117" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C117" s="18" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="118" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C118" s="18" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="119" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C119" s="18" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="120" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C120" s="18" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="121" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C121" s="18" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="122" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C122" s="17" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="123" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C123" s="18" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="124" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C124" s="18" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="125" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C125" s="18" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="126" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C126" s="18" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="127" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C127" s="18" t="s">
+        <v>137</v>
+      </c>
     </row>
     <row r="128" spans="3:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C128" s="23"/>
-      <c r="D128" s="23"/>
+      <c r="C128" s="26" t="s">
+        <v>138</v>
+      </c>
+      <c r="D128" s="26"/>
     </row>
     <row r="129" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="C129" s="23"/>
-      <c r="D129" s="23"/>
+      <c r="C129" s="26" t="s">
+        <v>139</v>
+      </c>
+      <c r="D129" s="26"/>
+    </row>
+    <row r="130" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="C130" s="18" t="s">
+        <v>140</v>
+      </c>
     </row>
     <row r="143" spans="2:12" ht="26.25" x14ac:dyDescent="0.4">
       <c r="B143" s="24"/>
-      <c r="E143" s="26"/>
-      <c r="F143" s="26"/>
-      <c r="G143" s="26"/>
-      <c r="H143" s="26"/>
-      <c r="I143" s="26"/>
-      <c r="J143" s="26"/>
-      <c r="K143" s="26"/>
-      <c r="L143" s="26"/>
+      <c r="E143" s="27"/>
+      <c r="F143" s="27"/>
+      <c r="G143" s="27"/>
+      <c r="H143" s="27"/>
+      <c r="I143" s="27"/>
+      <c r="J143" s="27"/>
+      <c r="K143" s="27"/>
+      <c r="L143" s="27"/>
     </row>
     <row r="144" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="E144" s="27"/>
+      <c r="E144" s="28"/>
       <c r="F144" s="28"/>
       <c r="G144" s="28"/>
       <c r="H144" s="28"/>
@@ -1079,7 +2033,7 @@
       <c r="L144" s="28"/>
     </row>
     <row r="145" spans="5:12" x14ac:dyDescent="0.25">
-      <c r="E145" s="27"/>
+      <c r="E145" s="28"/>
       <c r="F145" s="28"/>
       <c r="G145" s="28"/>
       <c r="H145" s="28"/>
@@ -1129,7 +2083,7 @@
       <c r="L149" s="28"/>
     </row>
     <row r="150" spans="5:12" x14ac:dyDescent="0.25">
-      <c r="E150" s="27"/>
+      <c r="E150" s="28"/>
       <c r="F150" s="28"/>
       <c r="G150" s="28"/>
       <c r="H150" s="28"/>
@@ -1179,7 +2133,7 @@
       <c r="L154" s="28"/>
     </row>
     <row r="155" spans="5:12" x14ac:dyDescent="0.25">
-      <c r="E155" s="27"/>
+      <c r="E155" s="28"/>
       <c r="F155" s="28"/>
       <c r="G155" s="28"/>
       <c r="H155" s="28"/>
@@ -1229,7 +2183,7 @@
       <c r="L159" s="28"/>
     </row>
     <row r="160" spans="5:12" x14ac:dyDescent="0.25">
-      <c r="E160" s="27"/>
+      <c r="E160" s="28"/>
       <c r="F160" s="28"/>
       <c r="G160" s="28"/>
       <c r="H160" s="28"/>

</xml_diff>

<commit_message>
GĐ 1-7: Cài Laravel Breeze V2.3.7 để thiết lập hệ thống đăng ký, đăng nhập, và xác thực cơ bản cho ứng dụng Laravel.
</commit_message>
<xml_diff>
--- a/Schedule-Note.xlsx
+++ b/Schedule-Note.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\task-manager-laravel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{266B8F02-CB50-480E-A754-D10B4FA4F85C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D977E63-1C37-44E2-B62E-5F41E386BA99}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Schedule" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="165">
   <si>
     <t>STT</t>
   </si>
@@ -478,9 +478,6 @@
     <t>tạo 8 file (folder default chứa file mặc định của laravel)</t>
   </si>
   <si>
-    <t>9 file migrations (11 table, 3 table tạo từ file User)</t>
-  </si>
-  <si>
     <t>Bảng</t>
   </si>
   <si>
@@ -524,6 +521,16 @@
   </si>
   <si>
     <t>Phân loại Seeder / Factory cho từng bảng</t>
+  </si>
+  <si>
+    <t>7 file migrations (9 table, 3 table tạo từ file User)</t>
+  </si>
+  <si>
+    <t>php artisan make:seeder UserSeeder; php artisan db:seed --class=UserSeeder</t>
+  </si>
+  <si>
+    <t>Breeze laravel: composer require laravel/breeze --dev
+php artisan breeze:install (tạo frontend Blade mặc định)</t>
   </si>
 </sst>
 </file>
@@ -727,7 +734,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -787,15 +794,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="16" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -813,6 +811,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -861,7 +860,9 @@
     <xf numFmtId="49" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -869,7 +870,7 @@
   <dxfs count="2">
     <dxf>
       <font>
-        <color rgb="FFFF0000"/>
+        <color rgb="FF00B050"/>
       </font>
       <fill>
         <patternFill>
@@ -879,7 +880,7 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF00B050"/>
+        <color rgb="FFFF0000"/>
       </font>
       <fill>
         <patternFill>
@@ -1026,6 +1027,50 @@
         <a:xfrm>
           <a:off x="4857750" y="7181850"/>
           <a:ext cx="10440857" cy="5811061"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>132</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>1087362</xdr:colOff>
+      <xdr:row>150</xdr:row>
+      <xdr:rowOff>133867</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9AD82A92-BC15-441A-9DCF-4BD2A2C2D4FC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1266825" y="25260300"/>
+          <a:ext cx="10831437" cy="3705742"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1322,7 +1367,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:K20"/>
+  <dimension ref="A2:K19"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.28515625" style="8" bestFit="1" customWidth="1"/>
@@ -1333,37 +1378,37 @@
     <col min="6" max="7" width="9.140625" style="8"/>
     <col min="8" max="8" width="32.7109375" style="8" customWidth="1"/>
     <col min="9" max="9" width="10.140625" style="8" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="59.140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="70.5703125" style="8" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="49.5703125" style="8" customWidth="1"/>
     <col min="12" max="16384" width="9.140625" style="8"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:11" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="37" t="s">
+      <c r="A2" s="35" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="37"/>
-      <c r="C2" s="37"/>
-      <c r="D2" s="37"/>
-      <c r="E2" s="37"/>
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="35"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
-      <c r="D3" s="38" t="s">
+      <c r="D3" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="E3" s="38"/>
+      <c r="E3" s="36"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
-      <c r="D4" s="38" t="s">
+      <c r="D4" s="36" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="38"/>
+      <c r="E4" s="36"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -1371,12 +1416,12 @@
       <c r="C5" s="1"/>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
-      <c r="H5" s="39" t="s">
+      <c r="H5" s="37" t="s">
         <v>26</v>
       </c>
-      <c r="I5" s="40"/>
-      <c r="J5" s="40"/>
-      <c r="K5" s="40"/>
+      <c r="I5" s="38"/>
+      <c r="J5" s="38"/>
+      <c r="K5" s="38"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
@@ -1414,19 +1459,19 @@
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="41">
+      <c r="A7" s="39">
         <v>1</v>
       </c>
-      <c r="B7" s="44" t="s">
+      <c r="B7" s="42" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="50" t="s">
+      <c r="C7" s="48" t="s">
         <v>30</v>
       </c>
-      <c r="D7" s="44" t="s">
+      <c r="D7" s="42" t="s">
         <v>32</v>
       </c>
-      <c r="E7" s="47" t="s">
+      <c r="E7" s="45" t="s">
         <v>25</v>
       </c>
       <c r="F7" s="21"/>
@@ -1443,11 +1488,11 @@
       <c r="K7" s="22"/>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" s="42"/>
-      <c r="B8" s="45"/>
-      <c r="C8" s="51"/>
-      <c r="D8" s="45"/>
-      <c r="E8" s="48"/>
+      <c r="A8" s="40"/>
+      <c r="B8" s="43"/>
+      <c r="C8" s="49"/>
+      <c r="D8" s="43"/>
+      <c r="E8" s="46"/>
       <c r="F8" s="21"/>
       <c r="G8" s="21"/>
       <c r="H8" s="24" t="s">
@@ -1464,62 +1509,70 @@
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9" s="42"/>
-      <c r="B9" s="45"/>
-      <c r="C9" s="51"/>
-      <c r="D9" s="45"/>
-      <c r="E9" s="48"/>
+      <c r="A9" s="40"/>
+      <c r="B9" s="43"/>
+      <c r="C9" s="49"/>
+      <c r="D9" s="43"/>
+      <c r="E9" s="46"/>
       <c r="F9" s="21"/>
       <c r="G9" s="21"/>
       <c r="H9" s="24" t="s">
         <v>139</v>
       </c>
       <c r="I9" s="25">
-        <v>45843</v>
+        <v>45844</v>
       </c>
       <c r="J9" s="24" t="s">
         <v>145</v>
       </c>
       <c r="K9" s="24" t="s">
-        <v>147</v>
+        <v>162</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" s="42"/>
-      <c r="B10" s="45"/>
-      <c r="C10" s="51"/>
-      <c r="D10" s="45"/>
-      <c r="E10" s="48"/>
+      <c r="A10" s="40"/>
+      <c r="B10" s="43"/>
+      <c r="C10" s="49"/>
+      <c r="D10" s="43"/>
+      <c r="E10" s="46"/>
       <c r="F10" s="21"/>
       <c r="G10" s="21"/>
       <c r="H10" s="24" t="s">
         <v>140</v>
       </c>
-      <c r="I10" s="26"/>
-      <c r="J10" s="27"/>
+      <c r="I10" s="25">
+        <v>45845</v>
+      </c>
+      <c r="J10" s="27" t="s">
+        <v>163</v>
+      </c>
       <c r="K10" s="27"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A11" s="42"/>
-      <c r="B11" s="45"/>
-      <c r="C11" s="51"/>
-      <c r="D11" s="45"/>
-      <c r="E11" s="48"/>
+    <row r="11" spans="1:11" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A11" s="40"/>
+      <c r="B11" s="43"/>
+      <c r="C11" s="49"/>
+      <c r="D11" s="43"/>
+      <c r="E11" s="46"/>
       <c r="F11" s="21"/>
       <c r="G11" s="21"/>
       <c r="H11" s="24" t="s">
         <v>141</v>
       </c>
-      <c r="I11" s="26"/>
-      <c r="J11" s="27"/>
+      <c r="I11" s="25">
+        <v>45845</v>
+      </c>
+      <c r="J11" s="51" t="s">
+        <v>164</v>
+      </c>
       <c r="K11" s="27"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A12" s="43"/>
-      <c r="B12" s="46"/>
-      <c r="C12" s="52"/>
-      <c r="D12" s="46"/>
-      <c r="E12" s="49"/>
+      <c r="A12" s="41"/>
+      <c r="B12" s="44"/>
+      <c r="C12" s="50"/>
+      <c r="D12" s="44"/>
+      <c r="E12" s="47"/>
       <c r="F12" s="21"/>
       <c r="G12" s="21"/>
       <c r="H12" s="24" t="s">
@@ -1529,18 +1582,18 @@
       <c r="J12" s="27"/>
       <c r="K12" s="27"/>
     </row>
-    <row r="13" spans="1:11" ht="63" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>32</v>
+        <v>11</v>
       </c>
       <c r="E13" s="7" t="s">
         <v>25</v>
@@ -1555,31 +1608,31 @@
         <v>3</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E14" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="H14" s="31"/>
-      <c r="I14" s="32"/>
-      <c r="J14" s="32"/>
-      <c r="K14" s="33"/>
+      <c r="H14" s="28"/>
+      <c r="I14" s="29"/>
+      <c r="J14" s="29"/>
+      <c r="K14" s="30"/>
     </row>
     <row r="15" spans="1:11" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="D15" s="3" t="s">
         <v>8</v>
@@ -1587,65 +1640,65 @@
       <c r="E15" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="H15" s="31"/>
-      <c r="I15" s="32"/>
-      <c r="J15" s="32"/>
-      <c r="K15" s="33"/>
+      <c r="H15" s="28"/>
+      <c r="I15" s="29"/>
+      <c r="J15" s="29"/>
+      <c r="K15" s="30"/>
     </row>
     <row r="16" spans="1:11" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E16" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="H16" s="31"/>
-      <c r="I16" s="32"/>
-      <c r="J16" s="32"/>
-      <c r="K16" s="33"/>
+      <c r="H16" s="28"/>
+      <c r="I16" s="29"/>
+      <c r="J16" s="29"/>
+      <c r="K16" s="30"/>
     </row>
     <row r="17" spans="1:11" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A17" s="3">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="E17" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="H17" s="31"/>
-      <c r="I17" s="32"/>
-      <c r="J17" s="32"/>
-      <c r="K17" s="33"/>
-    </row>
-    <row r="18" spans="1:11" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="H17" s="28"/>
+      <c r="I17" s="29"/>
+      <c r="J17" s="29"/>
+      <c r="K17" s="30"/>
+    </row>
+    <row r="18" spans="1:11" ht="44.25" x14ac:dyDescent="0.25">
       <c r="A18" s="3">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="E18" s="7" t="s">
         <v>25</v>
@@ -1655,29 +1708,8 @@
       <c r="J18" s="32"/>
       <c r="K18" s="33"/>
     </row>
-    <row r="19" spans="1:11" ht="44.25" x14ac:dyDescent="0.25">
-      <c r="A19" s="3">
-        <v>7</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="C19" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E19" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="H19" s="34"/>
-      <c r="I19" s="35"/>
-      <c r="J19" s="35"/>
-      <c r="K19" s="36"/>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="C20" s="9"/>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="C19" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -1692,11 +1724,11 @@
     <mergeCell ref="C7:C12"/>
   </mergeCells>
   <conditionalFormatting sqref="E1:E1048576">
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
+      <formula>$G$6</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
       <formula>$F$6</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
-      <formula>$G$6</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2055,8 +2087,8 @@
       <c r="C70" s="13" t="s">
         <v>81</v>
       </c>
-      <c r="D70" s="53" t="s">
-        <v>162</v>
+      <c r="D70" s="34" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="71" spans="3:6" x14ac:dyDescent="0.25">
@@ -2064,13 +2096,13 @@
         <v>82</v>
       </c>
       <c r="D71" s="13" t="s">
+        <v>147</v>
+      </c>
+      <c r="E71" s="13" t="s">
         <v>148</v>
       </c>
-      <c r="E71" s="13" t="s">
+      <c r="F71" s="13" t="s">
         <v>149</v>
-      </c>
-      <c r="F71" s="13" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="72" spans="3:6" x14ac:dyDescent="0.25">
@@ -2078,13 +2110,13 @@
         <v>83</v>
       </c>
       <c r="D72" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="E72" s="13" t="s">
         <v>151</v>
       </c>
-      <c r="E72" s="13" t="s">
+      <c r="F72" s="13" t="s">
         <v>152</v>
-      </c>
-      <c r="F72" s="13" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="73" spans="3:6" x14ac:dyDescent="0.25">
@@ -2092,13 +2124,13 @@
         <v>77</v>
       </c>
       <c r="D73" s="13" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E73" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="F73" s="13" t="s">
         <v>152</v>
-      </c>
-      <c r="F73" s="13" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="74" spans="3:6" x14ac:dyDescent="0.25">
@@ -2106,13 +2138,13 @@
         <v>84</v>
       </c>
       <c r="D74" s="13" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E74" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="F74" s="13" t="s">
         <v>152</v>
-      </c>
-      <c r="F74" s="13" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="75" spans="3:6" x14ac:dyDescent="0.25">
@@ -2120,13 +2152,13 @@
         <v>85</v>
       </c>
       <c r="D75" s="13" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E75" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="F75" s="13" t="s">
         <v>152</v>
-      </c>
-      <c r="F75" s="13" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="76" spans="3:6" x14ac:dyDescent="0.25">
@@ -2134,13 +2166,13 @@
         <v>86</v>
       </c>
       <c r="D76" s="13" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E76" s="13" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F76" s="13" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="77" spans="3:6" x14ac:dyDescent="0.25">
@@ -2148,13 +2180,13 @@
         <v>87</v>
       </c>
       <c r="D77" s="13" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E77" s="13" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F77" s="13" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="78" spans="3:6" x14ac:dyDescent="0.25">
@@ -2162,13 +2194,13 @@
         <v>88</v>
       </c>
       <c r="D78" s="13" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="E78" s="13" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F78" s="13" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="79" spans="3:6" x14ac:dyDescent="0.25">
@@ -2176,13 +2208,13 @@
         <v>89</v>
       </c>
       <c r="D79" s="13" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="E79" s="13" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F79" s="13" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="80" spans="3:6" x14ac:dyDescent="0.25">
@@ -2190,13 +2222,13 @@
         <v>90</v>
       </c>
       <c r="D80" s="13" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E80" s="13" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F80" s="13" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="81" spans="3:3" x14ac:dyDescent="0.25">
@@ -2445,6 +2477,11 @@
     <row r="130" spans="2:12" x14ac:dyDescent="0.25">
       <c r="C130" s="13" t="s">
         <v>136</v>
+      </c>
+    </row>
+    <row r="131" spans="2:12" ht="26.25" x14ac:dyDescent="0.4">
+      <c r="B131" s="11">
+        <v>45845</v>
       </c>
     </row>
     <row r="143" spans="2:12" ht="26.25" x14ac:dyDescent="0.4">

</xml_diff>